<commit_message>
📊 [auto] Economic data update — 2026-09-11 16:49 UTC
</commit_message>
<xml_diff>
--- a/reports/excel/MacroPulse_2026-09-11.xlsx
+++ b/reports/excel/MacroPulse_2026-09-11.xlsx
@@ -651,7 +651,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MacroPulse 總體經濟指標報告　　生成時間：2026-09-11 00:23 UTC</t>
+          <t>MacroPulse 總體經濟指標報告　　生成時間：2026-09-11 16:49 UTC</t>
         </is>
       </c>
     </row>
@@ -740,12 +740,12 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>332.8</t>
+          <t>334.1</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>3.54%</t>
+          <t>3.71%</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>0.07%</t>
+          <t>0.40%</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -802,12 +802,12 @@
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>336.8</t>
+          <t>337.8</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="H4" s="9" t="inlineStr">
         <is>
-          <t>2.79%</t>
+          <t>2.76%</t>
         </is>
       </c>
       <c r="I4" s="7" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
-          <t>0.21%</t>
+          <t>0.29%</t>
         </is>
       </c>
       <c r="K4" s="7" t="inlineStr">
@@ -2866,7 +2866,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>🔥 通膨指標　歷史數據　　生成時間：2026-09-11 00:23 UTC</t>
+          <t>🔥 通膨指標　歷史數據　　生成時間：2026-09-11 16:49 UTC</t>
         </is>
       </c>
     </row>
@@ -14555,32 +14555,32 @@
       </c>
       <c r="B123" s="20" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C123" s="20" t="inlineStr">
-        <is>
-          <t>N/A</t>
+          <t>334.1</t>
+        </is>
+      </c>
+      <c r="C123" s="6" t="inlineStr">
+        <is>
+          <t>3.71%</t>
         </is>
       </c>
       <c r="D123" s="20" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0.40%</t>
         </is>
       </c>
       <c r="E123" s="20" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F123" s="20" t="inlineStr">
-        <is>
-          <t>N/A</t>
+          <t>337.8</t>
+        </is>
+      </c>
+      <c r="F123" s="9" t="inlineStr">
+        <is>
+          <t>2.76%</t>
         </is>
       </c>
       <c r="G123" s="20" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0.29%</t>
         </is>
       </c>
       <c r="H123" s="20" t="inlineStr">
@@ -14688,7 +14688,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>📈 經濟成長　歷史數據　　生成時間：2026-09-11 00:23 UTC</t>
+          <t>📈 經濟成長　歷史數據　　生成時間：2026-09-11 16:49 UTC</t>
         </is>
       </c>
     </row>
@@ -24692,7 +24692,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>👷 勞動市場　歷史數據　　生成時間：2026-09-11 00:23 UTC</t>
+          <t>👷 勞動市場　歷史數據　　生成時間：2026-09-11 16:49 UTC</t>
         </is>
       </c>
     </row>
@@ -36517,7 +36517,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>🏦 利率與債券　歷史數據　　生成時間：2026-09-11 00:23 UTC</t>
+          <t>🏦 利率與債券　歷史數據　　生成時間：2026-09-11 16:49 UTC</t>
         </is>
       </c>
     </row>
@@ -48336,7 +48336,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>💭 信心指數　歷史數據　　生成時間：2026-09-11 00:23 UTC</t>
+          <t>💭 信心指數　歷史數據　　生成時間：2026-09-11 16:49 UTC</t>
         </is>
       </c>
     </row>
@@ -56513,7 +56513,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>⚠️ 信用與違約　歷史數據　　生成時間：2026-09-11 00:23 UTC</t>
+          <t>⚠️ 信用與違約　歷史數據　　生成時間：2026-09-11 16:49 UTC</t>
         </is>
       </c>
     </row>
@@ -59729,7 +59729,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>🏠 房市　歷史數據　　生成時間：2026-09-11 00:23 UTC</t>
+          <t>🏠 房市　歷史數據　　生成時間：2026-09-11 16:49 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>